<commit_message>
updated positive test for ECOCCUR=Y
</commit_message>
<xml_diff>
--- a/rules/CORE-000004/negative/01/data/unit-test-coreid-CG0101-negative.xlsx
+++ b/rules/CORE-000004/negative/01/data/unit-test-coreid-CG0101-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silvia.Faini\CORE\Rule_Authoring\core-contributor\rules\CORE-000004\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45546B7-A822-4E37-BE69-2AC480E6440D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A322DE3B-A387-402B-9E03-0C6531DB0B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="90">
   <si>
     <t>Product</t>
   </si>
@@ -70,6 +70,12 @@
     <t>Record</t>
   </si>
   <si>
+    <t>ECOCCUR</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
     <t>ECDOSE</t>
   </si>
   <si>
@@ -91,9 +97,6 @@
     <t>ECPRESP</t>
   </si>
   <si>
-    <t>ECOCCUR</t>
-  </si>
-  <si>
     <t>ECDOSU</t>
   </si>
   <si>
@@ -266,9 +269,6 @@
   </si>
   <si>
     <t>PLACEBO</t>
-  </si>
-  <si>
-    <t>N</t>
   </si>
   <si>
     <t/>
@@ -299,7 +299,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -322,8 +322,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -340,12 +344,6 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -359,13 +357,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -763,15 +762,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -807,10 +799,10 @@
         <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -827,7 +819,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3" s="2">
         <v>0</v>
@@ -847,10 +839,10 @@
         <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -867,7 +859,7 @@
         <v>17</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -887,10 +879,10 @@
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -907,7 +899,7 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -927,10 +919,10 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -947,60 +939,16 @@
         <v>19</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F9" s="2">
         <v>-10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="2">
-        <v>5</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="2">
-        <v>20</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="2">
-        <v>5</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="2">
-        <v>20</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F11">
-    <sortCondition ref="A2:A11"/>
-    <sortCondition ref="D2:D11"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1012,188 +960,188 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="J3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="P3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
@@ -1260,58 +1208,58 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H5" s="2">
         <v>5</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N5" s="2">
         <v>10.8</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="S5" s="2">
         <v>1</v>
@@ -1322,58 +1270,58 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D6" s="2">
         <v>2</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2">
         <v>5</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N6" s="2">
         <v>10.8</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="S6" s="2">
         <v>2</v>
@@ -1384,58 +1332,58 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="2">
         <v>3</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H7" s="2">
         <v>5</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N7" s="2">
         <v>10.8</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="S7" s="2">
         <v>3</v>
@@ -1446,58 +1394,58 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" s="2">
         <v>4</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2">
         <v>5</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N8" s="2">
         <v>10.8</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S8" s="2">
         <v>4</v>
@@ -1508,58 +1456,58 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D9" s="2">
         <v>5</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H9" s="2">
         <v>5</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N9" s="2">
         <v>10.8</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="S9" s="2">
         <v>5</v>
@@ -1570,58 +1518,58 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D10" s="2">
         <v>6</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H10" s="2">
         <v>5</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N10" s="2">
         <v>10.8</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="S10" s="2">
         <v>6</v>
@@ -1632,58 +1580,58 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D11" s="2">
         <v>7</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2">
         <v>5</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N11" s="2">
         <v>10.8</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S11" s="2">
         <v>7</v>
@@ -1694,58 +1642,58 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" s="2">
         <v>8</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2">
         <v>5</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N12" s="2">
         <v>10.8</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S12" s="2">
         <v>8</v>
@@ -1756,58 +1704,58 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D13" s="2">
         <v>9</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H13" s="2">
         <v>5</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N13" s="2">
         <v>10.8</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S13" s="2">
         <v>9</v>
@@ -1818,58 +1766,58 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D14" s="2">
         <v>10</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H14" s="2">
         <v>5</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N14" s="2">
         <v>10.8</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S14" s="2">
         <v>10</v>
@@ -1880,40 +1828,40 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D15" s="2">
         <v>122</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="H15" s="4">
         <v>0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>83</v>
@@ -1922,10 +1870,10 @@
         <v>0</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>84</v>
@@ -1942,40 +1890,40 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2">
         <v>123</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="H16" s="2">
         <v>20</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>83</v>
@@ -1984,10 +1932,10 @@
         <v>0</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>85</v>
@@ -2004,40 +1952,40 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D17" s="2">
         <v>124</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="H17" s="4">
         <v>0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>83</v>
@@ -2046,10 +1994,10 @@
         <v>0</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>86</v>
@@ -2066,40 +2014,40 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" s="2">
         <v>125</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="H18" s="4">
         <v>0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>83</v>
@@ -2108,10 +2056,10 @@
         <v>0</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>87</v>
@@ -2128,40 +2076,40 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" s="2">
         <v>126</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="H19" s="4">
         <v>-10</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>83</v>
@@ -2170,10 +2118,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>88</v>
@@ -2190,40 +2138,38 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="2">
         <v>127</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="H20" s="4">
-        <v>0</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H20" s="6"/>
       <c r="I20" s="2" t="s">
         <v>82</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>83</v>
@@ -2232,10 +2178,10 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>89</v>
@@ -2253,7 +2199,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:T15 A20:G20 A17:G17 I17:T17 A18:G18 I18:T18 A19:G19 I19:T19 I20:T20 A16:G16 I16:T16" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:T14 A20:G20 A15:H19 J15:T19 I20:T20" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reviewed rule, updated YAML and test data. Reran validation, no more unmatched validations
</commit_message>
<xml_diff>
--- a/rules/CORE-000004/negative/01/data/unit-test-coreid-CG0101-negative.xlsx
+++ b/rules/CORE-000004/negative/01/data/unit-test-coreid-CG0101-negative.xlsx
@@ -886,9 +886,7 @@
       <c r="E4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="8">
-        <v>0</v>
-      </c>
+      <c r="F4" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="7">
@@ -946,9 +944,7 @@
       <c r="E7" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="8">
-        <v>0</v>
-      </c>
+      <c r="F7" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="7">

</xml_diff>